<commit_message>
added road restriction lines back
</commit_message>
<xml_diff>
--- a/data/excel/restriction_list.xlsx
+++ b/data/excel/restriction_list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3a9e347b09434a31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R38de1accff034929"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11531,6 +11531,978 @@
         <x:v>被災路肩復旧・路盤入替 / 追加表示用データ</x:v>
       </x:c>
     </x:row>
+    <x:row r="387">
+      <x:c r="A387" t="str">
+        <x:v>R-081</x:v>
+      </x:c>
+      <x:c r="B387" t="str">
+        <x:v>宝立地区 通行止め 周辺規制01</x:v>
+      </x:c>
+      <x:c r="C387" t="str"/>
+      <x:c r="D387" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E387" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F387" s="3" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="G387" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H387" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I387" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="388">
+      <x:c r="A388" t="str">
+        <x:v>R-082</x:v>
+      </x:c>
+      <x:c r="B388" t="str">
+        <x:v>宝立地区 道路規制 周辺規制02</x:v>
+      </x:c>
+      <x:c r="C388" t="str"/>
+      <x:c r="D388" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E388" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F388" s="3" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="G388" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H388" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I388" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="389">
+      <x:c r="A389" t="str">
+        <x:v>R-083</x:v>
+      </x:c>
+      <x:c r="B389" t="str">
+        <x:v>宝立地区 通行止め 周辺規制03</x:v>
+      </x:c>
+      <x:c r="C389" t="str"/>
+      <x:c r="D389" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E389" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F389" s="3" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="G389" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H389" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I389" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390">
+      <x:c r="A390" t="str">
+        <x:v>R-084</x:v>
+      </x:c>
+      <x:c r="B390" t="str">
+        <x:v>宝立地区 道路規制 周辺規制04</x:v>
+      </x:c>
+      <x:c r="C390" t="str"/>
+      <x:c r="D390" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E390" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F390" s="3" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="G390" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H390" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I390" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391">
+      <x:c r="A391" t="str">
+        <x:v>R-085</x:v>
+      </x:c>
+      <x:c r="B391" t="str">
+        <x:v>宝立地区 通行止め 周辺規制05</x:v>
+      </x:c>
+      <x:c r="C391" t="str"/>
+      <x:c r="D391" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E391" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F391" s="3" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G391" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H391" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I391" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392">
+      <x:c r="A392" t="str">
+        <x:v>R-086</x:v>
+      </x:c>
+      <x:c r="B392" t="str">
+        <x:v>宝立地区 道路規制 周辺規制06</x:v>
+      </x:c>
+      <x:c r="C392" t="str"/>
+      <x:c r="D392" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E392" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F392" s="3" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="G392" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H392" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I392" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393">
+      <x:c r="A393" t="str">
+        <x:v>R-167</x:v>
+      </x:c>
+      <x:c r="B393" t="str">
+        <x:v>飯田地区 通行止め 周辺規制07</x:v>
+      </x:c>
+      <x:c r="C393" t="str"/>
+      <x:c r="D393" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E393" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F393" s="3" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="G393" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H393" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I393" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394">
+      <x:c r="A394" t="str">
+        <x:v>R-168</x:v>
+      </x:c>
+      <x:c r="B394" t="str">
+        <x:v>飯田地区 道路規制 周辺規制08</x:v>
+      </x:c>
+      <x:c r="C394" t="str"/>
+      <x:c r="D394" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E394" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F394" s="3" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="G394" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H394" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I394" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395">
+      <x:c r="A395" t="str">
+        <x:v>R-169</x:v>
+      </x:c>
+      <x:c r="B395" t="str">
+        <x:v>飯田地区 通行止め 周辺規制09</x:v>
+      </x:c>
+      <x:c r="C395" t="str"/>
+      <x:c r="D395" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E395" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F395" s="3" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="G395" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H395" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I395" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396">
+      <x:c r="A396" t="str">
+        <x:v>R-170</x:v>
+      </x:c>
+      <x:c r="B396" t="str">
+        <x:v>飯田地区 道路規制 周辺規制10</x:v>
+      </x:c>
+      <x:c r="C396" t="str"/>
+      <x:c r="D396" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E396" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F396" s="3" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G396" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H396" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I396" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397">
+      <x:c r="A397" t="str">
+        <x:v>R-171</x:v>
+      </x:c>
+      <x:c r="B397" t="str">
+        <x:v>飯田地区 通行止め 周辺規制11</x:v>
+      </x:c>
+      <x:c r="C397" t="str"/>
+      <x:c r="D397" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E397" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F397" s="3" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="G397" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H397" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I397" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398">
+      <x:c r="A398" t="str">
+        <x:v>R-172</x:v>
+      </x:c>
+      <x:c r="B398" t="str">
+        <x:v>飯田地区 道路規制 周辺規制12</x:v>
+      </x:c>
+      <x:c r="C398" t="str"/>
+      <x:c r="D398" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E398" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F398" s="3" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="G398" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H398" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I398" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399">
+      <x:c r="A399" t="str">
+        <x:v>R-941</x:v>
+      </x:c>
+      <x:c r="B399" t="str">
+        <x:v>正院地区 通行止め 周辺規制13</x:v>
+      </x:c>
+      <x:c r="C399" t="str"/>
+      <x:c r="D399" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E399" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F399" s="3" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="G399" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H399" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I399" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400">
+      <x:c r="A400" t="str">
+        <x:v>R-942</x:v>
+      </x:c>
+      <x:c r="B400" t="str">
+        <x:v>正院地区 道路規制 周辺規制14</x:v>
+      </x:c>
+      <x:c r="C400" t="str"/>
+      <x:c r="D400" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E400" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F400" s="3" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="G400" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H400" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I400" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401">
+      <x:c r="A401" t="str">
+        <x:v>R-943</x:v>
+      </x:c>
+      <x:c r="B401" t="str">
+        <x:v>正院地区 通行止め 周辺規制15</x:v>
+      </x:c>
+      <x:c r="C401" t="str"/>
+      <x:c r="D401" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E401" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F401" s="3" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G401" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H401" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I401" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402">
+      <x:c r="A402" t="str">
+        <x:v>R-944</x:v>
+      </x:c>
+      <x:c r="B402" t="str">
+        <x:v>正院地区 道路規制 周辺規制16</x:v>
+      </x:c>
+      <x:c r="C402" t="str"/>
+      <x:c r="D402" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E402" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F402" s="3" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="G402" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H402" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I402" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="403">
+      <x:c r="A403" t="str">
+        <x:v>R-945</x:v>
+      </x:c>
+      <x:c r="B403" t="str">
+        <x:v>正院地区 通行止め 周辺規制17</x:v>
+      </x:c>
+      <x:c r="C403" t="str"/>
+      <x:c r="D403" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E403" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F403" s="3" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="G403" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H403" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I403" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404">
+      <x:c r="A404" t="str">
+        <x:v>R-946</x:v>
+      </x:c>
+      <x:c r="B404" t="str">
+        <x:v>正院地区 道路規制 周辺規制18</x:v>
+      </x:c>
+      <x:c r="C404" t="str"/>
+      <x:c r="D404" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E404" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F404" s="3" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="G404" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H404" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I404" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="405">
+      <x:c r="A405" t="str">
+        <x:v>R-1169</x:v>
+      </x:c>
+      <x:c r="B405" t="str">
+        <x:v>直地区 通行止め 周辺規制19</x:v>
+      </x:c>
+      <x:c r="C405" t="str"/>
+      <x:c r="D405" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E405" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F405" s="3" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="G405" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H405" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I405" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="406">
+      <x:c r="A406" t="str">
+        <x:v>R-1170</x:v>
+      </x:c>
+      <x:c r="B406" t="str">
+        <x:v>直地区 道路規制 周辺規制20</x:v>
+      </x:c>
+      <x:c r="C406" t="str"/>
+      <x:c r="D406" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E406" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F406" s="3" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G406" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H406" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I406" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407">
+      <x:c r="A407" t="str">
+        <x:v>R-1171</x:v>
+      </x:c>
+      <x:c r="B407" t="str">
+        <x:v>直地区 通行止め 周辺規制21</x:v>
+      </x:c>
+      <x:c r="C407" t="str"/>
+      <x:c r="D407" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E407" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F407" s="3" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="G407" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H407" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I407" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408">
+      <x:c r="A408" t="str">
+        <x:v>R-1172</x:v>
+      </x:c>
+      <x:c r="B408" t="str">
+        <x:v>直地区 道路規制 周辺規制22</x:v>
+      </x:c>
+      <x:c r="C408" t="str"/>
+      <x:c r="D408" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E408" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F408" s="3" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="G408" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H408" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I408" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="409">
+      <x:c r="A409" t="str">
+        <x:v>R-1173</x:v>
+      </x:c>
+      <x:c r="B409" t="str">
+        <x:v>直地区 通行止め 周辺規制23</x:v>
+      </x:c>
+      <x:c r="C409" t="str"/>
+      <x:c r="D409" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E409" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F409" s="3" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="G409" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H409" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I409" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410">
+      <x:c r="A410" t="str">
+        <x:v>R-1174</x:v>
+      </x:c>
+      <x:c r="B410" t="str">
+        <x:v>直地区 道路規制 周辺規制24</x:v>
+      </x:c>
+      <x:c r="C410" t="str"/>
+      <x:c r="D410" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E410" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F410" s="3" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="G410" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H410" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I410" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411">
+      <x:c r="A411" t="str">
+        <x:v>R-1673</x:v>
+      </x:c>
+      <x:c r="B411" t="str">
+        <x:v>蛸島地区 通行止め 周辺規制25</x:v>
+      </x:c>
+      <x:c r="C411" t="str"/>
+      <x:c r="D411" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E411" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F411" s="3" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G411" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H411" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I411" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412">
+      <x:c r="A412" t="str">
+        <x:v>R-1674</x:v>
+      </x:c>
+      <x:c r="B412" t="str">
+        <x:v>蛸島地区 道路規制 周辺規制26</x:v>
+      </x:c>
+      <x:c r="C412" t="str"/>
+      <x:c r="D412" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E412" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F412" s="3" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="G412" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H412" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I412" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413">
+      <x:c r="A413" t="str">
+        <x:v>R-1675</x:v>
+      </x:c>
+      <x:c r="B413" t="str">
+        <x:v>蛸島地区 通行止め 周辺規制27</x:v>
+      </x:c>
+      <x:c r="C413" t="str"/>
+      <x:c r="D413" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E413" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F413" s="3" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="G413" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H413" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I413" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414">
+      <x:c r="A414" t="str">
+        <x:v>R-1676</x:v>
+      </x:c>
+      <x:c r="B414" t="str">
+        <x:v>蛸島地区 道路規制 周辺規制28</x:v>
+      </x:c>
+      <x:c r="C414" t="str"/>
+      <x:c r="D414" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E414" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F414" s="3" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="G414" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H414" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I414" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415">
+      <x:c r="A415" t="str">
+        <x:v>R-1677</x:v>
+      </x:c>
+      <x:c r="B415" t="str">
+        <x:v>蛸島地区 通行止め 周辺規制29</x:v>
+      </x:c>
+      <x:c r="C415" t="str"/>
+      <x:c r="D415" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E415" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F415" s="3" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="G415" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H415" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I415" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416">
+      <x:c r="A416" t="str">
+        <x:v>R-1678</x:v>
+      </x:c>
+      <x:c r="B416" t="str">
+        <x:v>蛸島地区 道路規制 周辺規制30</x:v>
+      </x:c>
+      <x:c r="C416" t="str"/>
+      <x:c r="D416" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E416" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F416" s="3" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G416" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H416" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I416" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417">
+      <x:c r="A417" t="str">
+        <x:v>R-2457</x:v>
+      </x:c>
+      <x:c r="B417" t="str">
+        <x:v>上戸地区 通行止め 周辺規制31</x:v>
+      </x:c>
+      <x:c r="C417" t="str"/>
+      <x:c r="D417" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E417" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F417" s="3" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="G417" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H417" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I417" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418">
+      <x:c r="A418" t="str">
+        <x:v>R-2458</x:v>
+      </x:c>
+      <x:c r="B418" t="str">
+        <x:v>上戸地区 道路規制 周辺規制32</x:v>
+      </x:c>
+      <x:c r="C418" t="str"/>
+      <x:c r="D418" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E418" s="3" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="F418" s="3" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="G418" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H418" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I418" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419">
+      <x:c r="A419" t="str">
+        <x:v>R-2459</x:v>
+      </x:c>
+      <x:c r="B419" t="str">
+        <x:v>上戸地区 通行止め 周辺規制33</x:v>
+      </x:c>
+      <x:c r="C419" t="str"/>
+      <x:c r="D419" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E419" s="3" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="F419" s="3" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="G419" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H419" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I419" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420">
+      <x:c r="A420" t="str">
+        <x:v>R-2460</x:v>
+      </x:c>
+      <x:c r="B420" t="str">
+        <x:v>上戸地区 道路規制 周辺規制34</x:v>
+      </x:c>
+      <x:c r="C420" t="str"/>
+      <x:c r="D420" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E420" s="3" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="F420" s="3" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="G420" t="str">
+        <x:v>珠洲市</x:v>
+      </x:c>
+      <x:c r="H420" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I420" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421">
+      <x:c r="A421" t="str">
+        <x:v>R-2461</x:v>
+      </x:c>
+      <x:c r="B421" t="str">
+        <x:v>上戸地区 通行止め 周辺規制35</x:v>
+      </x:c>
+      <x:c r="C421" t="str"/>
+      <x:c r="D421" t="str">
+        <x:v>通行止め</x:v>
+      </x:c>
+      <x:c r="E421" s="3" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="F421" s="3" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G421" t="str">
+        <x:v>交通誘導班</x:v>
+      </x:c>
+      <x:c r="H421" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I421" t="str">
+        <x:v>工事区域周辺の安全確保のため一時通行止め / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422">
+      <x:c r="A422" t="str">
+        <x:v>R-2462</x:v>
+      </x:c>
+      <x:c r="B422" t="str">
+        <x:v>上戸地区 道路規制 周辺規制36</x:v>
+      </x:c>
+      <x:c r="C422" t="str"/>
+      <x:c r="D422" t="str">
+        <x:v>道路規制</x:v>
+      </x:c>
+      <x:c r="E422" s="3" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="F422" s="3" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="G422" t="str">
+        <x:v>道路管理班</x:v>
+      </x:c>
+      <x:c r="H422" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I422" t="str">
+        <x:v>工事区域周辺の誘導・速度抑制区間 / 工事エリア周辺の交通規制</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>